<commit_message>
Extra parts highlighted in BOM #22
</commit_message>
<xml_diff>
--- a/BOM/eSpark-BOM-IoT-Speaker.xlsx
+++ b/BOM/eSpark-BOM-IoT-Speaker.xlsx
@@ -5,7 +5,7 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\smartmasjid-hardware\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Faizan\GitHub\smartmasjid-hardware\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -1024,7 +1024,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="[$-409]h:mm:ss\ AM/PM;@"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.0000"/>
@@ -1222,7 +1222,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1250,6 +1250,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1545,7 +1551,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="88">
+  <cellXfs count="99">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1788,6 +1794,39 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="21" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="6" borderId="17" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="18" fillId="6" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="6" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="18" fillId="6" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="19" fillId="6" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="18" fillId="6" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1832,7 +1871,7 @@
         <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1886,7 +1925,7 @@
         <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1940,7 +1979,7 @@
         <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1994,7 +2033,7 @@
         <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2048,7 +2087,7 @@
         <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -16079,50 +16118,50 @@
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
-      <c r="C22" s="52" t="s">
+      <c r="C22" s="88" t="s">
         <v>14</v>
       </c>
-      <c r="D22" s="71" t="s">
+      <c r="D22" s="94" t="s">
         <v>30</v>
       </c>
-      <c r="E22" s="49" t="s">
+      <c r="E22" s="89" t="s">
         <v>51</v>
       </c>
-      <c r="F22" s="49" t="s">
+      <c r="F22" s="89" t="s">
         <v>162</v>
       </c>
-      <c r="G22" s="49" t="s">
+      <c r="G22" s="89" t="s">
         <v>91</v>
       </c>
-      <c r="H22" s="49" t="s">
+      <c r="H22" s="89" t="s">
         <v>110</v>
       </c>
-      <c r="I22" s="49" t="s">
-        <v>160</v>
-      </c>
-      <c r="J22" s="49" t="s">
+      <c r="I22" s="89" t="s">
+        <v>160</v>
+      </c>
+      <c r="J22" s="89" t="s">
         <v>129</v>
       </c>
-      <c r="K22" s="49" t="s">
-        <v>160</v>
-      </c>
-      <c r="L22" s="49">
+      <c r="K22" s="89" t="s">
+        <v>160</v>
+      </c>
+      <c r="L22" s="89">
         <v>1</v>
       </c>
-      <c r="M22" s="37">
+      <c r="M22" s="90">
         <f t="shared" si="1"/>
         <v>3000</v>
       </c>
-      <c r="N22" s="37">
+      <c r="N22" s="90">
         <v>3020</v>
       </c>
-      <c r="O22" s="64" t="s">
-        <v>165</v>
-      </c>
-      <c r="P22" s="50">
+      <c r="O22" s="91" t="s">
+        <v>165</v>
+      </c>
+      <c r="P22" s="92">
         <v>1.8800000000000001E-2</v>
       </c>
-      <c r="Q22" s="38">
+      <c r="Q22" s="96">
         <f>P22*N22</f>
         <v>56.776000000000003</v>
       </c>
@@ -16634,50 +16673,50 @@
         <f t="shared" si="0"/>
         <v>23</v>
       </c>
-      <c r="C32" s="52" t="s">
+      <c r="C32" s="88" t="s">
         <v>21</v>
       </c>
-      <c r="D32" s="71" t="s">
+      <c r="D32" s="94" t="s">
         <v>226</v>
       </c>
-      <c r="E32" s="49" t="s">
+      <c r="E32" s="89" t="s">
         <v>57</v>
       </c>
-      <c r="F32" s="49" t="s">
+      <c r="F32" s="89" t="s">
         <v>75</v>
       </c>
-      <c r="G32" s="49" t="s">
+      <c r="G32" s="89" t="s">
         <v>95</v>
       </c>
-      <c r="H32" s="49" t="s">
+      <c r="H32" s="89" t="s">
         <v>114</v>
       </c>
-      <c r="I32" s="49" t="s">
-        <v>160</v>
-      </c>
-      <c r="J32" s="49" t="s">
+      <c r="I32" s="89" t="s">
+        <v>160</v>
+      </c>
+      <c r="J32" s="89" t="s">
         <v>132</v>
       </c>
-      <c r="K32" s="37" t="s">
-        <v>160</v>
-      </c>
-      <c r="L32" s="49">
+      <c r="K32" s="90" t="s">
+        <v>160</v>
+      </c>
+      <c r="L32" s="89">
         <v>2</v>
       </c>
-      <c r="M32" s="37">
+      <c r="M32" s="90">
         <f t="shared" si="1"/>
         <v>6000</v>
       </c>
-      <c r="N32" s="37">
+      <c r="N32" s="90">
         <v>6020</v>
       </c>
-      <c r="O32" s="64" t="s">
-        <v>165</v>
-      </c>
-      <c r="P32" s="50">
+      <c r="O32" s="91" t="s">
+        <v>165</v>
+      </c>
+      <c r="P32" s="92">
         <v>1.9199999999999998E-2</v>
       </c>
-      <c r="Q32" s="76">
+      <c r="Q32" s="98">
         <f>P32*N32</f>
         <v>115.58399999999999</v>
       </c>
@@ -16690,50 +16729,50 @@
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
-      <c r="C33" s="51" t="s">
+      <c r="C33" s="93" t="s">
         <v>21</v>
       </c>
-      <c r="D33" s="37" t="s">
+      <c r="D33" s="90" t="s">
         <v>227</v>
       </c>
-      <c r="E33" s="37" t="s">
+      <c r="E33" s="90" t="s">
         <v>58</v>
       </c>
-      <c r="F33" s="37" t="s">
+      <c r="F33" s="90" t="s">
         <v>76</v>
       </c>
-      <c r="G33" s="37" t="s">
+      <c r="G33" s="90" t="s">
         <v>96</v>
       </c>
-      <c r="H33" s="37" t="s">
+      <c r="H33" s="90" t="s">
         <v>115</v>
       </c>
-      <c r="I33" s="37" t="s">
-        <v>160</v>
-      </c>
-      <c r="J33" s="37" t="s">
+      <c r="I33" s="90" t="s">
+        <v>160</v>
+      </c>
+      <c r="J33" s="90" t="s">
         <v>133</v>
       </c>
-      <c r="K33" s="37" t="s">
-        <v>160</v>
-      </c>
-      <c r="L33" s="37">
+      <c r="K33" s="90" t="s">
+        <v>160</v>
+      </c>
+      <c r="L33" s="90">
         <v>3</v>
       </c>
-      <c r="M33" s="37">
+      <c r="M33" s="90">
         <f t="shared" si="1"/>
         <v>9000</v>
       </c>
-      <c r="N33" s="71">
+      <c r="N33" s="94">
         <v>9020</v>
       </c>
-      <c r="O33" s="63" t="s">
-        <v>165</v>
-      </c>
-      <c r="P33" s="38">
+      <c r="O33" s="95" t="s">
+        <v>165</v>
+      </c>
+      <c r="P33" s="96">
         <v>1.5599999999999999E-2</v>
       </c>
-      <c r="Q33" s="74">
+      <c r="Q33" s="97">
         <f>P33*N33</f>
         <v>140.71199999999999</v>
       </c>
@@ -17975,50 +18014,50 @@
         <f t="shared" si="0"/>
         <v>47</v>
       </c>
-      <c r="C56" s="52" t="s">
+      <c r="C56" s="88" t="s">
         <v>25</v>
       </c>
-      <c r="D56" s="49" t="s">
+      <c r="D56" s="89" t="s">
         <v>180</v>
       </c>
-      <c r="E56" s="49" t="s">
+      <c r="E56" s="89" t="s">
         <v>287</v>
       </c>
-      <c r="F56" s="49" t="s">
+      <c r="F56" s="89" t="s">
         <v>288</v>
       </c>
-      <c r="G56" s="49" t="s">
+      <c r="G56" s="89" t="s">
         <v>289</v>
       </c>
-      <c r="H56" s="49" t="s">
+      <c r="H56" s="89" t="s">
         <v>117</v>
       </c>
-      <c r="I56" s="49" t="s">
-        <v>160</v>
-      </c>
-      <c r="J56" s="49" t="s">
+      <c r="I56" s="89" t="s">
+        <v>160</v>
+      </c>
+      <c r="J56" s="89" t="s">
         <v>290</v>
       </c>
-      <c r="K56" s="49" t="s">
-        <v>160</v>
-      </c>
-      <c r="L56" s="49">
+      <c r="K56" s="89" t="s">
+        <v>160</v>
+      </c>
+      <c r="L56" s="89">
         <v>1</v>
       </c>
-      <c r="M56" s="37">
+      <c r="M56" s="90">
         <f t="shared" si="1"/>
         <v>3000</v>
       </c>
-      <c r="N56" s="37">
+      <c r="N56" s="90">
         <v>3005</v>
       </c>
-      <c r="O56" s="64" t="s">
-        <v>165</v>
-      </c>
-      <c r="P56" s="50">
+      <c r="O56" s="91" t="s">
+        <v>165</v>
+      </c>
+      <c r="P56" s="92">
         <v>7.2400000000000006E-2</v>
       </c>
-      <c r="Q56" s="50">
+      <c r="Q56" s="92">
         <f t="shared" ref="Q56" si="23">P56*N56</f>
         <v>217.56200000000001</v>
       </c>

</xml_diff>